<commit_message>
Auto-save: 5 file(s) — 2026-09-29 09:48
</commit_message>
<xml_diff>
--- a/Notes/2026-09-29-xloop-blog-content-plan-q2.xlsx
+++ b/Notes/2026-09-29-xloop-blog-content-plan-q2.xlsx
@@ -1,15 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8370F2-B5D9-4FC4-991B-DD922974B78C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="12105" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Master Content Plan" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Funnel Overview" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="ICP Matrix" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="SEO-AEO-GEO" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Blog Outlines" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Summary Dashboard" state="visible" r:id="rId9"/>
+    <sheet name="Master Content Plan" sheetId="1" r:id="rId1"/>
+    <sheet name="Funnel Overview" sheetId="2" r:id="rId2"/>
+    <sheet name="ICP Matrix" sheetId="3" r:id="rId3"/>
+    <sheet name="SEO-AEO-GEO" sheetId="4" r:id="rId4"/>
+    <sheet name="Blog Outlines" sheetId="5" r:id="rId5"/>
+    <sheet name="Summary Dashboard" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -102,7 +106,7 @@
     <t>Others explain the obligations. We show what a non-intrusive IT/OT audit looks like on a live plant, from a delivered 30 MW wind IPP audit, written executive-first with clause detail below.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what the NEPRA Security of IT and OT Regulations 2022 require, in 50 words
+    <t>1. Intro: what the NEPRA Security of IT and OT Regulations 2022 require, in 50 words
 2. Who must comply (generation, transmission, distribution licensees)
 3. The obligations in plain language: security policy, risk assessment, IT/OT segregation, incident reporting (major incidents within 72 hours; breaches quarterly)
 4. What an IT/OT audit covers: governance, risk and vulnerability, SCADA/DCS/PLC/RTU/HMI, network segregation
@@ -125,7 +129,7 @@
     <t>Article + FAQPage</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: Pakistan (Karachi, Lahore, Islamabad power sector)
+    <t>GEO: Pakistan (Karachi, Lahore, Islamabad power sector)
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. Quote SRO 1708(I)/2022 exactly. Link to the NEPRA landing page, never compete with it. Never "NEPRA-approved".</t>
   </si>
   <si>
@@ -168,7 +172,7 @@
     <t>A checklist in the buyer's own words, tied to a free self-serve assessment with results before any form. Pakistani peers sell readiness only as consulting.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what "AI-ready data" means, answered in 50 words
+    <t>1. Intro: what "AI-ready data" means, answered in 50 words
 2. Why AI projects stall on data, not models
 3. The 10-point checklist: sources, definitions, duplicates, gaps, ownership, lineage, access, security, volume, freshness
 4. How to score yourself (simple 0–2 scale table)
@@ -191,7 +195,7 @@
     <t>Article + HowTo + FAQPage</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, US, UK, Pakistan
+    <t>GEO: UAE, Saudi Arabia, US, UK, Pakistan
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. Make the checklist an HTML list/table (AI engines extract lists). Link the Readiness Assessment above the fold.</t>
   </si>
   <si>
@@ -225,7 +229,7 @@
     <t>Written by an ISO 42001 Lead Auditor, not a tool vendor. Adds what regulators in Pakistan and the GCC expect (SBP direction on responsible AI, National AI Policy 2025) that US-centric guides skip. Security framed as the accelerator, not fear.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what enterprise AI security covers, in 50 words
+    <t>1. Intro: what enterprise AI security covers, in 50 words
 2. The five areas: visibility of AI use, data protection, model and prompt security, agent access, governance
 3. The risks that are new with AI (prompt injection, data leakage through retrieval, over-permissioned agents)
 4. What your existing pentest and SOC do and don't cover
@@ -245,7 +249,7 @@
     <t>enterprise AI security · secure enterprise AI, AI security for enterprises, AI security strategy for enterprises, generative AI security, AI governance</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, Pakistan, US
+    <t>GEO: UAE, Saudi Arabia, Pakistan, US
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. GSC: "enterprise ai security" 718 impr. at pos. 52 + 3 variants (~1,100 impr.). H1 and first sentence must contain the exact phrase.</t>
   </si>
   <si>
@@ -267,7 +271,7 @@
     <t>Quality as an architecture decision (checks in the pipeline, not in spreadsheets), from a named architect. Exact-query rewrite for a page that ranks at 73.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what AI data quality is, in 50 words
+    <t>1. Intro: what AI data quality is, in 50 words
 2. The six dimensions: accuracy, completeness, consistency, timeliness, uniqueness, validity
 3. How bad data shows up in AI (wrong answers, bias, hallucinated "facts")
 4. Measuring quality before a model depends on it
@@ -287,7 +291,7 @@
     <t>AI data quality · data quality for AI, AI and data quality, data quality AI, data quality management</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, US, UK, South Africa
+    <t>GEO: UAE, Saudi Arabia, US, UK, South Africa
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. GSC: "ai data quality" 207 impr. at pos. 73, "ai for data quality" 74, "data quality for ai" 52.</t>
   </si>
   <si>
@@ -309,7 +313,7 @@
     <t>"Find it without banning everything." Practical detection steps plus an approved-alternatives approach, instead of the usual "ban ChatGPT" take.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what shadow AI is, in 50 words
+    <t>1. Intro: what shadow AI is, in 50 words
 2. Why it happens (people trying to work faster)
 3. The real risk: what data goes in
 4. How to find it: network and SaaS logs, expense data, vendor AI features, asking teams
@@ -329,7 +333,7 @@
     <t>what is shadow AI · shadow AI risks, shadow AI detection, unapproved AI tools, employee ChatGPT use policy</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, Pakistan, US, UK
+    <t>GEO: UAE, Saudi Arabia, Pakistan, US, UK
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram.</t>
   </si>
   <si>
@@ -351,7 +355,7 @@
     <t>A real consolidation (SAP ERP + SAP BW + app databases into Snowflake), vendor-neutral and honest about limits (not real-time). Vendor content is platform-first.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: why dashboards disagree, in 50 words
+    <t>1. Intro: why dashboards disagree, in 50 words
 2. The usual causes: different sources, different definitions, manual extracts
 3. What a single source of truth is (and isn't)
 4. Warehouse vs lake vs lakehouse, briefly
@@ -371,7 +375,7 @@
     <t>single source of truth data · why reports don't match, data warehouse vs lakehouse, medallion architecture, SAP to Snowflake</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: South Africa, UAE, Saudi Arabia, US, UK
+    <t>GEO: South Africa, UAE, Saudi Arabia, US, UK
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. Never "real-time" or "data pulled manually" (CTO correction).</t>
   </si>
   <si>
@@ -393,7 +397,7 @@
     <t>A plain side-by-side for CISOs plus what an AI red-team exercise actually involves. Most content is vendor tooling or academic.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: the difference in 50 words
+    <t>1. Intro: the difference in 50 words
 2. What a penetration test checks
 3. What AI red teaming checks (prompts, models, agents, training data, outputs)
 4. Side-by-side comparison table
@@ -413,7 +417,7 @@
     <t>AI red teaming vs penetration testing · what is AI red teaming, LLM red teaming, AI security testing, red teaming generative AI</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, US, UK, Pakistan
+    <t>GEO: UAE, Saudi Arabia, US, UK, Pakistan
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. No client red-team findings without permission (claim B1).</t>
   </si>
   <si>
@@ -435,7 +439,7 @@
     <t>Workload-first sizing from engineers who run it, not cloud-vendor marketing. Page ranks 7.2 with 0 clicks: fix intent match.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: choose by workload, not the demo, in 50 words
+    <t>1. Intro: choose by workload, not the demo, in 50 words
 2. Four questions: peak volume, latency, model size, data location
 3. Managed AI services vs self-hosted models
 4. GPU vs CPU for inference
@@ -455,7 +459,7 @@
     <t>infrastructure for generative AI workloads · GenAI infrastructure, GPU vs CPU inference, AI infrastructure cost, scalable AI infrastructure</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, US, UK
+    <t>GEO: UAE, Saudi Arabia, US, UK
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. GSC: 3,564 impr., 0 clicks, pos. 7.2.</t>
   </si>
   <si>
@@ -480,7 +484,7 @@
     <t>Written by a certified ISO 42001 Lead Auditor: what auditors ask first. Strong expertise signal for search and AI engines.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what ISO/IEC 42001 is, in 50 words
+    <t>1. Intro: what ISO/IEC 42001 is, in 50 words
 2. Who it applies to
 3. What it requires: AI policy, roles, risk and impact assessment, controls, monitoring, improvement
 4. How it relates to ISO 27001
@@ -500,7 +504,7 @@
     <t>ISO 42001 explained · ISO 42001 requirements, AI management system, ISO 42001 vs ISO 27001, ISO 42001 certification</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, Pakistan, UK
+    <t>GEO: UAE, Saudi Arabia, Pakistan, UK
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. Lead Auditor credential is individual. Never "xLoop is ISO 42001 certified".</t>
   </si>
   <si>
@@ -525,7 +529,7 @@
     <t>Practical "prepare for SBP expectations" section, plus delivered FS work (LLM assistant for an AMC, mobile banking security, COBOL → Java). Page ranks 7.1 with 0 clicks.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: where AI works in banking, in 50 words
+    <t>1. Intro: where AI works in banking, in 50 words
 2. Use cases that work: service, fraud, onboarding, credit, research assistants
 3. What it takes: data, security, governance
 4. Regulators: what SBP has signaled (verify status on publish day)
@@ -545,7 +549,7 @@
     <t>AI in banking · AI in asset management, AI banking Pakistan, State Bank of Pakistan AI, AI fraud detection banking, GenAI financial services</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: Pakistan, UAE, Saudi Arabia
+    <t>GEO: Pakistan, UAE, Saudi Arabia
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. Named clients allowed: Alfalah Investments, HBL Asset Management.</t>
   </si>
   <si>
@@ -579,7 +583,7 @@
     <t>An engineering account at real scale (over 1 billion records, 4,000+ frontline workers). Existing content is academic or startup news.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what national-scale health platforms need, in 50 words
+    <t>1. Intro: what national-scale health platforms need, in 50 words
 2. Offline-first apps for frontline workers
 3. A data layer built to grow
 4. Protecting patient data (security assessment lessons)
@@ -599,7 +603,7 @@
     <t>digital health platform at scale · health data platform, offline-first health app, scaling healthcare platform, patient data security</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: Pakistan, UAE, Saudi Arabia, Canada
+    <t>GEO: Pakistan, UAE, Saudi Arabia, Canada
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. Never name IRD, never mention WHO, never "Java 19".</t>
   </si>
   <si>
@@ -627,7 +631,7 @@
     <t>Data-first and vendor-neutral, with a real retailer story and honest limits. Highest-impression blog on the site (5,414).</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: how retailers use AI, in 50 words
+    <t>1. Intro: how retailers use AI, in 50 words
 2. Personalization
 3. Demand forecasting and inventory
 4. Pricing and promotions
@@ -647,7 +651,7 @@
     <t>AI in retail · AI retail optimization, hyper personalization in retail, AI inventory optimization, retail data platform</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: South Africa, UAE, Saudi Arabia, Pakistan
+    <t>GEO: South Africa, UAE, Saudi Arabia, Pakistan
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. GSC: 5,414 impr., pos. 12.8. Pick n Pay naming: confirm first.</t>
   </si>
   <si>
@@ -675,7 +679,7 @@
     <t>"Where to start", from building a container depot platform, against product pages from Oracle, Infor and Modula.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: how AI is used in warehouses and depots, in 50 words
+    <t>1. Intro: how AI is used in warehouses and depots, in 50 words
 2. Use cases: inspection, capacity planning, forecasting, task prioritization
 3. Why digitizing comes first
 4. Case: a cloud-native container depot platform (inspection, repairs, scheduling, invoicing, capacity)
@@ -695,7 +699,7 @@
     <t>AI in warehouse management · AI warehouse management use cases, container depot software, AI logistics operations, digital depot management</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: Pakistan, UAE, Saudi Arabia
+    <t>GEO: Pakistan, UAE, Saudi Arabia
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. GSC: 414 + 261 + 102 + 83 impr. across variants, pos. 18–60.</t>
   </si>
   <si>
@@ -723,7 +727,7 @@
     <t>Five things a PoC must prove (value, data, ownership, cost, risk), from delivery, not theory.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: why pilots stall, in 50 words
+    <t>1. Intro: why pilots stall, in 50 words
 2. The pilot trap
 3. The five things a PoC must prove
 4. Success measures agreed before the pilot
@@ -743,7 +747,7 @@
     <t>AI projects stuck in pilot · AI proof of concept, AI pilot to production, why AI projects fail</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, US, UK
+    <t>GEO: UAE, Saudi Arabia, US, UK
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. GSC: 842 impr., 0 clicks, pos. 16.</t>
   </si>
   <si>
@@ -768,7 +772,7 @@
     <t>Our real 11-stage architecture and named stack. Strongest technical-credibility asset we have.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what a production multi-agent system needs, in 50 words
+    <t>1. Intro: what a production multi-agent system needs, in 50 words
 2. When you need more than one agent
 3–7. The 11 stages (pull names from the AI deck): input guardrails, task decomposition, orchestration, tool and knowledge layers, reflection, human approval, observability…
 8. FAQ
@@ -784,7 +788,7 @@
     <t>multi-agent AI architecture · agentic AI architecture, AI agents in production, LangGraph architecture</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: US, UK, UAE
+    <t>GEO: US, UK, UAE
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. No partnership with Anthropic/OpenAI implied.</t>
   </si>
   <si>
@@ -806,7 +810,7 @@
     <t>A method, not unsourced ROI numbers. Conversational ROI queries already reach us at position 4.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what an AI business case must answer, in 50 words
+    <t>1. Intro: what an AI business case must answer, in 50 words
 2–8. The seven questions: process changed, today's measure, what good looks like, data, ownership, running cost, stop criteria
 9. CTA: take the Data &amp; AI Readiness Assessment</t>
   </si>
@@ -820,7 +824,7 @@
     <t>AI business case · AI ROI, how to calculate AI ROI, AI investment decision</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, US, UK, Pakistan
+    <t>GEO: UAE, Saudi Arabia, US, UK, Pakistan
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram.</t>
   </si>
   <si>
@@ -842,7 +846,7 @@
     <t>A point of view: the fundamentals are the same; choose by data residency, licenses and skills. Never name Microsoft Fabric.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: the short answer, in 50 words
+    <t>1. Intro: the short answer, in 50 words
 2. What both do well
 3. Where they differ
 4. Data residency
@@ -862,7 +866,7 @@
     <t>Snowflake vs Databricks · lakehouse platform comparison, Snowflake or Databricks for AI, data platform selection</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: US, UK, UAE, South Africa
+    <t>GEO: US, UK, UAE, South Africa
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram. Never mention Microsoft Fabric.</t>
   </si>
   <si>
@@ -884,7 +888,7 @@
     <t>Bridges both tracks: governance as the thing that lets GenAI touch real data safely.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: the minimum governance for GenAI, in 50 words
+    <t>1. Intro: the minimum governance for GenAI, in 50 words
 2. Classification
 3. Access that follows the user
 4. Lineage
@@ -904,7 +908,7 @@
     <t>data governance for generative AI · GenAI data governance, AI data access control, data classification AI</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: UAE, Saudi Arabia, US, UK
+    <t>GEO: UAE, Saudi Arabia, US, UK
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram.</t>
   </si>
   <si>
@@ -929,7 +933,7 @@
     <t>One plain example, then the controls that actually work. No fear-selling.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: what prompt injection is, in 50 words
+    <t>1. Intro: what prompt injection is, in 50 words
 2. A simple example
 3. Direct vs indirect injection
 4. Why filters alone fail
@@ -967,7 +971,7 @@
     <t>Built from a delivered engagement guiding a bank's apps toward PCI-DSS and State Bank compliance.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Intro: the layers, in 50 words
+    <t>1. Intro: the layers, in 50 words
 2. Reverse-engineering and API assessment
 3. Code obfuscation
 4. API authentication and encryption
@@ -987,7 +991,7 @@
     <t>mobile banking app security · banking app penetration testing, PCI-DSS mobile app, State Bank of Pakistan app security</t>
   </si>
   <si>
-    <t xml:space="preserve">GEO: Pakistan, UAE, Saudi Arabia
+    <t>GEO: Pakistan, UAE, Saudi Arabia
 AEO: H2s written as the questions buyers ask; answer each in the first 1–2 sentences. 40–60 word answer-first intro. FAQ block + FAQPage schema. Named expert author with credentials. One original table / checklist / diagram.</t>
   </si>
   <si>
@@ -1339,22 +1343,22 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd-mmm-yy"/>
+    <numFmt numFmtId="164" formatCode="dd\-mmm\-yy"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1368,19 +1372,19 @@
     </font>
     <font>
       <i/>
+      <sz val="9"/>
       <color rgb="FF888888"/>
-      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="18"/>
       <color rgb="FF1E3A5F"/>
-      <sz val="18"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF666666"/>
-      <sz val="11"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1499,7 +1503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1561,8 +1565,6 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1625,6 +1627,11 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1964,9 +1971,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -1991,7 +1998,7 @@
     <col min="21" max="21" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2056,7 +2063,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2121,7 +2128,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -2186,7 +2193,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2251,7 +2258,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2316,7 +2323,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2381,7 +2388,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2446,7 +2453,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -2511,7 +2518,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -2576,7 +2583,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -2641,7 +2648,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -2706,7 +2713,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -2771,7 +2778,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -2836,7 +2843,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="14" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -2901,7 +2908,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -2966,7 +2973,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -3031,7 +3038,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="17" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -3096,7 +3103,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -3161,7 +3168,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -3226,7 +3233,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3291,7 +3298,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" ht="140" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -3357,24 +3364,21 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U21"/>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="U10:U21">
-      <formula1>"Not started,Outline approved,Drafting,In review,Approved,Published,Refreshed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="U2:U21">
+  <autoFilter ref="A1:U21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="U2:U21" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not started,Outline approved,Drafting,In review,Approved,Published,Refreshed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -3384,7 +3388,7 @@
     <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>269</v>
       </c>
@@ -3404,7 +3408,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
         <v>23</v>
       </c>
@@ -3424,7 +3428,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>42</v>
       </c>
@@ -3444,7 +3448,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>58</v>
       </c>
@@ -3464,7 +3468,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
         <v>58</v>
       </c>
@@ -3484,7 +3488,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>58</v>
       </c>
@@ -3504,7 +3508,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>42</v>
       </c>
@@ -3524,7 +3528,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>42</v>
       </c>
@@ -3544,7 +3548,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>42</v>
       </c>
@@ -3564,7 +3568,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>58</v>
       </c>
@@ -3584,7 +3588,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
         <v>42</v>
       </c>
@@ -3604,7 +3608,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>58</v>
       </c>
@@ -3624,7 +3628,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>58</v>
       </c>
@@ -3644,7 +3648,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>58</v>
       </c>
@@ -3664,7 +3668,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
         <v>42</v>
       </c>
@@ -3684,7 +3688,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>42</v>
       </c>
@@ -3704,7 +3708,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
         <v>23</v>
       </c>
@@ -3724,7 +3728,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
         <v>42</v>
       </c>
@@ -3744,7 +3748,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>58</v>
       </c>
@@ -3764,7 +3768,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>58</v>
       </c>
@@ -3784,7 +3788,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>42</v>
       </c>
@@ -3805,16 +3809,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F21"/>
+  <autoFilter ref="A1:F21" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -3822,10 +3826,10 @@
     <col min="4" max="4" width="50" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="34" customWidth="1"/>
-    <col min="7" max="7" width="46" customWidth="1"/>
+    <col min="7" max="7" width="53" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3848,7 +3852,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="2" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -3871,7 +3875,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -3894,7 +3898,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -3917,7 +3921,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="54.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -3940,7 +3944,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -3963,7 +3967,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -3986,7 +3990,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -4009,7 +4013,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="9" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -4032,7 +4036,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -4055,7 +4059,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="11" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -4078,7 +4082,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="12" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -4101,7 +4105,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="13" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -4124,7 +4128,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="14" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -4147,7 +4151,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="15" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -4170,7 +4174,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="16" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -4193,7 +4197,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="17" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -4216,7 +4220,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="18" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -4239,7 +4243,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="19" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -4262,7 +4266,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="20" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -4285,7 +4289,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="21" ht="55" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -4309,16 +4313,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G21"/>
+  <autoFilter ref="A1:G21" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -4332,7 +4336,7 @@
     <col min="10" max="10" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4364,7 +4368,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="2" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -4396,7 +4400,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="3" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -4428,7 +4432,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="4" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -4460,7 +4464,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="5" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -4492,7 +4496,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="6" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -4524,7 +4528,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="7" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -4556,7 +4560,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="8" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -4588,7 +4592,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="9" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -4620,7 +4624,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="10" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -4652,7 +4656,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="11" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -4684,7 +4688,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="12" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -4716,7 +4720,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="13" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -4748,7 +4752,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="14" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -4780,7 +4784,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="15" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -4812,7 +4816,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="16" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -4844,7 +4848,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="17" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -4876,7 +4880,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="18" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -4908,7 +4912,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="19" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -4940,7 +4944,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="20" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -4972,7 +4976,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="21" ht="80" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="48" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -5005,16 +5009,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J21"/>
+  <autoFilter ref="A1:J21" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -5024,7 +5028,7 @@
     <col min="6" max="6" width="78" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5044,7 +5048,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="2" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -5064,7 +5068,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -5084,7 +5088,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -5104,7 +5108,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -5124,7 +5128,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -5144,7 +5148,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -5164,7 +5168,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -5184,7 +5188,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="9" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -5204,7 +5208,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="10" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -5224,7 +5228,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -5244,7 +5248,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="12" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -5264,7 +5268,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="13" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -5284,7 +5288,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -5304,7 +5308,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="15" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -5324,7 +5328,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="16" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -5344,7 +5348,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="17" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -5364,7 +5368,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="18" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -5384,7 +5388,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="19" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -5404,7 +5408,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="20" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -5424,7 +5428,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="21" ht="140" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="140.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -5445,16 +5449,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F21"/>
+  <autoFilter ref="A1:F21" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:I24"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
@@ -5465,380 +5469,380 @@
     <col min="9" max="9" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:9" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="42" t="s">
         <v>357</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="43" t="s">
         <v>358</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="21" t="s">
         <v>359</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="G4" s="21" t="s">
         <v>360</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="23" t="s">
+      <c r="I4" s="21" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+    <row r="5" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="25">
+      <c r="B5" s="23">
         <v>1</v>
       </c>
-      <c r="C5" s="25">
+      <c r="C5" s="23">
         <v>0</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="23">
         <v>0</v>
       </c>
-      <c r="E5" s="25">
+      <c r="E5" s="23">
         <v>1</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="44">
         <v>46300</v>
       </c>
-      <c r="H5" s="26" t="s">
+      <c r="H5" s="24" t="s">
         <v>34</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="6" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="B6" s="28">
+    <row r="6" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="26">
         <v>14</v>
       </c>
-      <c r="C6" s="28">
+      <c r="C6" s="26">
         <v>6</v>
       </c>
-      <c r="D6" s="28">
+      <c r="D6" s="26">
         <v>7</v>
       </c>
-      <c r="E6" s="28">
+      <c r="E6" s="26">
         <v>1</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="44">
         <v>46307</v>
       </c>
-      <c r="H6" s="29" t="s">
+      <c r="H6" s="27" t="s">
         <v>53</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="7" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="30" t="s">
+    <row r="7" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="B7" s="31">
+      <c r="B7" s="29">
         <v>2</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="29">
         <v>0</v>
       </c>
-      <c r="D7" s="31">
+      <c r="D7" s="29">
         <v>2</v>
       </c>
-      <c r="E7" s="31">
+      <c r="E7" s="29">
         <v>0</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="44">
         <v>46314</v>
       </c>
-      <c r="H7" s="26" t="s">
+      <c r="H7" s="24" t="s">
         <v>34</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
+    <row r="8" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="B8" s="33">
+      <c r="B8" s="31">
         <v>1</v>
       </c>
-      <c r="C8" s="33">
+      <c r="C8" s="31">
         <v>1</v>
       </c>
-      <c r="D8" s="33">
+      <c r="D8" s="31">
         <v>0</v>
       </c>
-      <c r="E8" s="33">
+      <c r="E8" s="31">
         <v>0</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="44">
         <v>46321</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="H8" s="27" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="9" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="34" t="s">
+    <row r="9" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="32" t="s">
         <v>164</v>
       </c>
-      <c r="B9" s="35">
+      <c r="B9" s="33">
         <v>1</v>
       </c>
-      <c r="C9" s="35">
+      <c r="C9" s="33">
         <v>1</v>
       </c>
-      <c r="D9" s="35">
+      <c r="D9" s="33">
         <v>0</v>
       </c>
-      <c r="E9" s="35">
+      <c r="E9" s="33">
         <v>0</v>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="44">
         <v>46328</v>
       </c>
-      <c r="H9" s="26" t="s">
+      <c r="H9" s="24" t="s">
         <v>34</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="10" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="36" t="s">
+    <row r="10" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="34" t="s">
         <v>177</v>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="35">
         <v>1</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="35">
         <v>1</v>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="35">
         <v>0</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="35">
         <v>0</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="44">
         <v>46335</v>
       </c>
-      <c r="H10" s="29" t="s">
+      <c r="H10" s="27" t="s">
         <v>53</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="38" t="s">
+    <row r="11" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="36" t="s">
         <v>368</v>
       </c>
-      <c r="B11" s="38">
+      <c r="B11" s="36">
         <v>20</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="36">
         <v>9</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="36">
         <v>9</v>
       </c>
-      <c r="E11" s="38">
+      <c r="E11" s="36">
         <v>2</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="44">
         <v>46342</v>
       </c>
-      <c r="H11" s="26" t="s">
+      <c r="H11" s="24" t="s">
         <v>34</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G12" s="6">
+    <row r="12" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G12" s="44">
         <v>46349</v>
       </c>
-      <c r="H12" s="29" t="s">
+      <c r="H12" s="27" t="s">
         <v>53</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="13" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G13" s="6">
+    <row r="13" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="44">
         <v>46356</v>
       </c>
-      <c r="H13" s="26" t="s">
+      <c r="H13" s="24" t="s">
         <v>34</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="14" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G14" s="6">
+    <row r="14" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G14" s="44">
         <v>46363</v>
       </c>
-      <c r="H14" s="39" t="s">
+      <c r="H14" s="37" t="s">
         <v>147</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="15" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G15" s="6">
+    <row r="15" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G15" s="44">
         <v>46370</v>
       </c>
-      <c r="H15" s="39" t="s">
+      <c r="H15" s="37" t="s">
         <v>162</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="16" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G16" s="6">
+    <row r="16" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G16" s="44">
         <v>46377</v>
       </c>
-      <c r="H16" s="39" t="s">
+      <c r="H16" s="37" t="s">
         <v>175</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="17" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G17" s="6">
+    <row r="17" spans="7:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G17" s="44">
         <v>46384</v>
       </c>
-      <c r="H17" s="39" t="s">
+      <c r="H17" s="37" t="s">
         <v>188</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="18" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G18" s="40" t="s">
+    <row r="18" spans="7:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G18" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="H18" s="41" t="s">
+      <c r="H18" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="I18" s="40" t="s">
+      <c r="I18" s="38" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G19" s="40" t="s">
+    <row r="19" spans="7:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G19" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="H19" s="41" t="s">
+      <c r="H19" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="I19" s="40" t="s">
+      <c r="I19" s="38" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="20" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G20" s="40" t="s">
+    <row r="20" spans="7:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G20" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="H20" s="41" t="s">
+      <c r="H20" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="I20" s="40" t="s">
+      <c r="I20" s="38" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="21" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G21" s="40" t="s">
+    <row r="21" spans="7:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G21" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="H21" s="41" t="s">
+      <c r="H21" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="I21" s="40" t="s">
+      <c r="I21" s="38" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G22" s="40" t="s">
+    <row r="22" spans="7:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G22" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="H22" s="42" t="s">
+      <c r="H22" s="40" t="s">
         <v>246</v>
       </c>
-      <c r="I22" s="40" t="s">
+      <c r="I22" s="38" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="23" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G23" s="40" t="s">
+    <row r="23" spans="7:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G23" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="H23" s="43" t="s">
+      <c r="H23" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="I23" s="40" t="s">
+      <c r="I23" s="38" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1" spans="7:9" x14ac:dyDescent="0.25">
-      <c r="G24" s="40" t="s">
+    <row r="24" spans="7:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G24" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="H24" s="43" t="s">
+      <c r="H24" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="I24" s="40" t="s">
+      <c r="I24" s="38" t="s">
         <v>382</v>
       </c>
     </row>
@@ -5848,6 +5852,6 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>